<commit_message>
Ajout de 4 machines (DX140LCR, DL220, DX360LC-0, Liebherr A914) + silhouette chargeuse
- nouveau type 'chargeuse' avec dessin LEGO dedie (godet frontal sur bras de levage)
- echelle des dessins elargie : 13 t -> 38 t, pour differencier les petites machines
- badge de type gere 3 cas (chenilles / pneus / chargeuse)
- generer_data.py reconnait chargeuse, DL###, LCR et Liebherr A###/R###
- Machines.xlsx complete (12 machines)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Machines.xlsx
+++ b/Machines.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -566,6 +566,70 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PELLE DX140LCR</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>28234</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CHARGEUSE DL220</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>28803</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>13</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>chargeuse</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PELLE DX360LC-0</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>28806</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PELLE LIEBHERR A914</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>28232</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>15</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>pneus</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>